<commit_message>
endret til bra struktur
</commit_message>
<xml_diff>
--- a/Grid/Enkel_nett_teste_qmaxmin.xlsx
+++ b/Grid/Enkel_nett_teste_qmaxmin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0348cbc925570652/Master/Kraftsystemer/Kraftsystemer-2/Grid/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_057EBA57FA9E57F87E476CE1F4362D3B786B1A4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{045EE466-EF47-4944-BB6C-1ACDD8B7D566}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_057EBA57FA9E57F87E476CE1F4362D3B786B1A4C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F09D82E2-886B-4E9E-A616-A203083450D0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bus" sheetId="1" r:id="rId1"/>
@@ -851,7 +851,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="H2">
         <v>62.492536000000001</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="H3">
         <v>63.385137599999993</v>

</xml_diff>